<commit_message>
Abcdefu (#15): FUCK YOU / FUCK OFF mehrmals je Chorus, Blinder 48,75 und 51,875; mehrere Zeitfenster je Ebene
- fxLayerWindow / fxTextWindow mit Platz (bis FX_LAYER_WINDOWS = 4 Fenster je Part), fades = false für ein
  Fenster ohne Ein-/Ausblenden, Ende darf hinter dem Part-Ende liegen (Ausblenden im nächsten Part)
- songgen.py: windows: in overlay und text (mit over), Einträge [von, bis], [von] oder {from, to, hard: true}
- Abcdefu: Text auf jedes F-U im Chorus und eine Viertel vor Chorus 2/3, 1,5 Takte voll + 0,5 Takte ausblenden;
  auf x,25 FUCK OFF; ab 80,75 weiß mit Rand statt ausgestanzt (über progFastBlingBling unsichtbar);
  neuer Blinder auf 48,75, Stopp-Blinder auf 51,875; case-Nummern jetzt fortlaufend (MIDI-Datei neu)
- Demo 92: Part 59 (drei Fenster in einem Part) am Anfang; Doku, Katalog, Plan, Skill, CLAUDE.md nachgezogen

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/Abcdefu_v1/quelle/struktur.xlsx
+++ b/songs/Abcdefu_v1/quelle/struktur.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="384" yWindow="384" windowWidth="27648" windowHeight="12276" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="468" yWindow="4572" windowWidth="27780" windowHeight="20436" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="abcdefu" sheetId="1" state="visible" r:id="rId1"/>
@@ -463,11 +463,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J371"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -571,7 +571,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>progBlack(7636, 5)
+          <t>progBlack(7636, 3)
 Alles schwarz bis zum Intro (die Matrix zeigt den Titel-Lauftext).</t>
         </is>
       </c>
@@ -770,7 +770,7 @@
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>progBlingBlingColoring(16909, 10, 3000)
+          <t>progBlingBlingColoring(16909, 4, 3000)
 Jedes Gerät füllt sich langsam LED für LED mit einer Farbe, alle 3 s kommt die nächste. Beginnt erst hier, nicht schon in der Pause.</t>
         </is>
       </c>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>progStrobo(1091, 15, 75, 255, 255, 255)
+          <t>progStrobo(1091, 5, 75, 255, 255, 255)
 Text (Matrix): "FUCK OFF": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
 2 Beats weißes Flimmern als Absprung in die Strophe (alter Effekt). Auf der Matrix steht dabei FUCK OFF schwarz ausgestanzt im Strobo: die Buchstaben bleiben dunkel, das Weiß blitzt drumherum.</t>
         </is>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>progPalette(15000, 1, 20)
+          <t>progPalette(15000, 1, 6)
 Alter Effekt: Regenbogen-Streifen mit harten Kanten laufen über die Geräte.</t>
         </is>
       </c>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>progMatrixScanner(15000, 25, 1)
+          <t>progMatrixScanner(15000, 7, 1)
 Alter Effekt: schneller Scanner, eine Leuchtlinie fährt hin und her.</t>
         </is>
       </c>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>progPalette(15000, 3, 30)
+          <t>progPalette(15000, 3, 8)
 Text (Matrix): "A B C D E": A 1 x, B 1 x, C 1 x, D 1 x, E 9 x 469 ms, ein Durchlauf 6097 ms (über der Szene)
    ab 12188 ms bis 14531 ms, darunter 15 %
 Alter Effekt: lila und grüne Balken. Ab Takt 6,5 des Parts (Beat 26) erscheinen auf der Matrix A, B, C, D, E in Weiß, je ein Viertel lang, über dem gedimmten Effekt.</t>
@@ -2394,7 +2394,7 @@
       <c r="G149" s="6" t="n"/>
       <c r="J149" s="7" t="n"/>
     </row>
-    <row r="150" collapsed="1" ht="28.8" customHeight="1">
+    <row r="150" ht="28.8" customHeight="1">
       <c r="A150" s="4" t="n">
         <v>37</v>
       </c>
@@ -2405,10 +2405,10 @@
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>progFullColors(15000, 35, 469)
-Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
-   ab 0 ms bis 5625 ms
-Alter Effekt: alle LEDs einfarbig, pro Beat eine neue Farbe. Auf der Matrix steht die ersten 3 Takte FUCK YOU schwarz ausgestanzt in der Farbfläche (Buchstaben dunkel, Farbe drumherum): hart an, steht ruhig ohne Pulsieren und ohne Ausblenden, nach 3 Takten hart weg.</t>
+          <t>progFullColors(15000, 9, 469)
+Text (Matrix): "FUCK_YOU FUCK_OFF": FUCK_YOU 29 x, FUCK_OFF 35 x 469 ms, ein Durchlauf 30016 ms (ausgestanzt aus der Szene)
+   Fenster 1: ab 0 ms bis 5625 ms, hart an und aus, Fenster 2: ab 7031 ms bis 10781 ms, Fenster 3: ab 13594 ms bis 17344 ms (blendet im nächsten Part aus), klingt 938 ms ab
+Alter Effekt: alle LEDs einfarbig, pro Beat eine neue Farbe. Auf der Matrix steht FUCK YOU schwarz ausgestanzt in der Farbfläche (Buchstaben dunkel, Farbe drumherum): die ersten 3 Takte hart an und hart weg, dann auf 40,75 FUCK YOU und auf 44,25 FUCK OFF, je 1,5 Takte voll und 0,5 Takte ausblendend.</t>
         </is>
       </c>
       <c r="D150" s="11" t="n"/>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="J150" s="7" t="n"/>
     </row>
-    <row r="151" hidden="1" outlineLevel="2">
+    <row r="151" outlineLevel="2">
       <c r="A151" s="4" t="n">
         <v>37.25</v>
       </c>
@@ -2438,7 +2438,7 @@
       <c r="G151" s="6" t="n"/>
       <c r="J151" s="7" t="n"/>
     </row>
-    <row r="152" hidden="1" outlineLevel="2">
+    <row r="152" outlineLevel="2">
       <c r="A152" s="4" t="n">
         <v>37.5</v>
       </c>
@@ -2450,7 +2450,7 @@
       <c r="G152" s="6" t="n"/>
       <c r="J152" s="7" t="n"/>
     </row>
-    <row r="153" hidden="1" outlineLevel="2">
+    <row r="153" outlineLevel="2">
       <c r="A153" s="4" t="n">
         <v>37.75</v>
       </c>
@@ -2462,7 +2462,7 @@
       <c r="G153" s="6" t="n"/>
       <c r="J153" s="7" t="n"/>
     </row>
-    <row r="154" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="154" outlineLevel="1" collapsed="1">
       <c r="A154" s="4" t="n">
         <v>38</v>
       </c>
@@ -2510,7 +2510,7 @@
       <c r="G157" s="6" t="n"/>
       <c r="J157" s="7" t="n"/>
     </row>
-    <row r="158" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="158" outlineLevel="1" collapsed="1">
       <c r="A158" s="4" t="n">
         <v>39</v>
       </c>
@@ -2558,7 +2558,7 @@
       <c r="G161" s="6" t="n"/>
       <c r="J161" s="7" t="n"/>
     </row>
-    <row r="162" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="162" outlineLevel="1">
       <c r="A162" s="4" t="n">
         <v>40</v>
       </c>
@@ -2570,7 +2570,7 @@
       <c r="G162" s="6" t="n"/>
       <c r="J162" s="7" t="n"/>
     </row>
-    <row r="163" hidden="1" outlineLevel="2">
+    <row r="163" outlineLevel="2">
       <c r="A163" s="4" t="n">
         <v>40.25</v>
       </c>
@@ -2582,7 +2582,7 @@
       <c r="G163" s="6" t="n"/>
       <c r="J163" s="7" t="n"/>
     </row>
-    <row r="164" hidden="1" outlineLevel="2">
+    <row r="164" outlineLevel="2">
       <c r="A164" s="4" t="n">
         <v>40.5</v>
       </c>
@@ -2594,19 +2594,28 @@
       <c r="G164" s="6" t="n"/>
       <c r="J164" s="7" t="n"/>
     </row>
-    <row r="165" hidden="1" outlineLevel="2">
+    <row r="165" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A165" s="4" t="n">
         <v>40.75</v>
       </c>
       <c r="B165" s="5" t="n"/>
-      <c r="C165" s="6" t="n"/>
-      <c r="D165" s="11" t="n"/>
+      <c r="C165" s="6" t="inlineStr">
+        <is>
+          <t>FUCK YOU schwarz ausgestanzt, 1,5 Takte voll, dann bis 42,75 ausblenden</t>
+        </is>
+      </c>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E165" s="10" t="n"/>
       <c r="F165" s="10" t="n"/>
       <c r="G165" s="6" t="n"/>
       <c r="J165" s="7" t="n"/>
     </row>
-    <row r="166" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="166" outlineLevel="1" collapsed="1">
       <c r="A166" s="4" t="n">
         <v>41</v>
       </c>
@@ -2654,7 +2663,7 @@
       <c r="G169" s="6" t="n"/>
       <c r="J169" s="7" t="n"/>
     </row>
-    <row r="170" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="170" outlineLevel="1" collapsed="1">
       <c r="A170" s="4" t="n">
         <v>42</v>
       </c>
@@ -2702,7 +2711,7 @@
       <c r="G173" s="6" t="n"/>
       <c r="J173" s="7" t="n"/>
     </row>
-    <row r="174" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="174" outlineLevel="1" collapsed="1">
       <c r="A174" s="4" t="n">
         <v>43</v>
       </c>
@@ -2750,7 +2759,7 @@
       <c r="G177" s="6" t="n"/>
       <c r="J177" s="7" t="n"/>
     </row>
-    <row r="178" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="178" outlineLevel="1">
       <c r="A178" s="4" t="n">
         <v>44</v>
       </c>
@@ -2762,19 +2771,28 @@
       <c r="G178" s="6" t="n"/>
       <c r="J178" s="7" t="n"/>
     </row>
-    <row r="179" hidden="1" outlineLevel="2">
+    <row r="179" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A179" s="4" t="n">
         <v>44.25</v>
       </c>
       <c r="B179" s="5" t="n"/>
-      <c r="C179" s="6" t="n"/>
-      <c r="D179" s="11" t="n"/>
+      <c r="C179" s="6" t="inlineStr">
+        <is>
+          <t>FUCK OFF schwarz ausgestanzt, 1,5 Takte voll, blendet im na na na na bis 46,25 aus</t>
+        </is>
+      </c>
+      <c r="D179" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK OFF": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E179" s="10" t="n"/>
       <c r="F179" s="10" t="n"/>
       <c r="G179" s="6" t="n"/>
       <c r="J179" s="7" t="n"/>
     </row>
-    <row r="180" hidden="1" outlineLevel="2">
+    <row r="180" outlineLevel="2">
       <c r="A180" s="4" t="n">
         <v>44.5</v>
       </c>
@@ -2786,7 +2804,7 @@
       <c r="G180" s="6" t="n"/>
       <c r="J180" s="7" t="n"/>
     </row>
-    <row r="181" hidden="1" outlineLevel="2">
+    <row r="181" outlineLevel="2">
       <c r="A181" s="4" t="n">
         <v>44.75</v>
       </c>
@@ -2798,7 +2816,7 @@
       <c r="G181" s="6" t="n"/>
       <c r="J181" s="7" t="n"/>
     </row>
-    <row r="182" collapsed="1" ht="28.8" customHeight="1">
+    <row r="182" ht="28.8" customHeight="1">
       <c r="A182" s="4" t="n">
         <v>45</v>
       </c>
@@ -2809,11 +2827,18 @@
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>progSternNeu(7500, 469, 40, 5, 26, 5, false, 4)
-Alter Effekt: drehender Stern, fest in der Mitte, Farbwechsel pro Beat.</t>
-        </is>
-      </c>
-      <c r="D182" s="12" t="n"/>
+          <t>progSternNeu(7500, 469, 10, 5, 26, 5, false, 4)
+Text (Matrix): "FUCK OFF": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+   Fenster 1: ab 0 ms bis 2344 ms, klingt 938 ms ab
+Ausgabe: Blinder voll bei Takt 48,75 = 7031 ms, 1172 ms lang, Blinder blendet in den 234 ms davor ein, 0 ms voll, 938 ms aus, Blinder liegt unter dem Text
+Alter Effekt: drehender Stern, fest in der Mitte, Farbwechsel pro Beat. Das FUCK OFF aus dem Chorus steht noch 3 Beats und blendet bis 46,25 aus. Auf 48,75 ein warmweißer Blinder, der bis 49,25 in die Strophe ausklingt.</t>
+        </is>
+      </c>
+      <c r="D182" s="12" t="inlineStr">
+        <is>
+          <t>text s.o.</t>
+        </is>
+      </c>
       <c r="E182" s="10" t="n">
         <v>4</v>
       </c>
@@ -2828,7 +2853,7 @@
       </c>
       <c r="J182" s="7" t="n"/>
     </row>
-    <row r="183" hidden="1" outlineLevel="2">
+    <row r="183" outlineLevel="2">
       <c r="A183" s="4" t="n">
         <v>45.25</v>
       </c>
@@ -2840,7 +2865,7 @@
       <c r="G183" s="6" t="n"/>
       <c r="J183" s="7" t="n"/>
     </row>
-    <row r="184" hidden="1" outlineLevel="2">
+    <row r="184" outlineLevel="2">
       <c r="A184" s="4" t="n">
         <v>45.5</v>
       </c>
@@ -2852,7 +2877,7 @@
       <c r="G184" s="6" t="n"/>
       <c r="J184" s="7" t="n"/>
     </row>
-    <row r="185" hidden="1" outlineLevel="2">
+    <row r="185" outlineLevel="2">
       <c r="A185" s="4" t="n">
         <v>45.75</v>
       </c>
@@ -2864,7 +2889,7 @@
       <c r="G185" s="6" t="n"/>
       <c r="J185" s="7" t="n"/>
     </row>
-    <row r="186" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="186" outlineLevel="1" collapsed="1">
       <c r="A186" s="4" t="n">
         <v>46</v>
       </c>
@@ -2912,7 +2937,7 @@
       <c r="G189" s="6" t="n"/>
       <c r="J189" s="7" t="n"/>
     </row>
-    <row r="190" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="190" outlineLevel="1" collapsed="1">
       <c r="A190" s="4" t="n">
         <v>47</v>
       </c>
@@ -2960,7 +2985,7 @@
       <c r="G193" s="6" t="n"/>
       <c r="J193" s="7" t="n"/>
     </row>
-    <row r="194" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="194" outlineLevel="1">
       <c r="A194" s="4" t="n">
         <v>48</v>
       </c>
@@ -2972,7 +2997,7 @@
       <c r="G194" s="6" t="n"/>
       <c r="J194" s="7" t="n"/>
     </row>
-    <row r="195" hidden="1" outlineLevel="2">
+    <row r="195" outlineLevel="2">
       <c r="A195" s="4" t="n">
         <v>48.25</v>
       </c>
@@ -2984,7 +3009,7 @@
       <c r="G195" s="6" t="n"/>
       <c r="J195" s="7" t="n"/>
     </row>
-    <row r="196" hidden="1" outlineLevel="2">
+    <row r="196" outlineLevel="2">
       <c r="A196" s="4" t="n">
         <v>48.5</v>
       </c>
@@ -2996,19 +3021,27 @@
       <c r="G196" s="6" t="n"/>
       <c r="J196" s="7" t="n"/>
     </row>
-    <row r="197" hidden="1" outlineLevel="2">
+    <row r="197" outlineLevel="2" ht="28.8" customHeight="1">
       <c r="A197" s="4" t="n">
         <v>48.75</v>
       </c>
       <c r="B197" s="5" t="n"/>
-      <c r="C197" s="6" t="n"/>
-      <c r="D197" s="12" t="n"/>
+      <c r="C197" s="6" t="inlineStr">
+        <is>
+          <t>Blinder (warmweiß, alle Geräte): blendet eine halbe Viertel ein, auf 48,75 voll, klingt bis 49,25 aus</t>
+        </is>
+      </c>
+      <c r="D197" s="12" t="inlineStr">
+        <is>
+          <t>Blinder einfügen (höhepunkt bei 48,74, fade out bis 49,25)</t>
+        </is>
+      </c>
       <c r="E197" s="10" t="n"/>
       <c r="F197" s="10" t="n"/>
       <c r="G197" s="6" t="n"/>
       <c r="J197" s="7" t="n"/>
     </row>
-    <row r="198" collapsed="1" ht="28.8" customHeight="1">
+    <row r="198" ht="28.8" customHeight="1">
       <c r="A198" s="4" t="n">
         <v>49</v>
       </c>
@@ -3019,8 +3052,9 @@
       </c>
       <c r="C198" s="6" t="inlineStr">
         <is>
-          <t>progBlingBlingColoring(5625, 45, 5000)
-Alter Effekt: langsames Füllen LED für LED, alle 5 s eine neue Farbe.</t>
+          <t>progBlingBlingColoring(5625, 11, 5000)
+Ausgabe: Blinder bei Takt 51,875 = 5391 ms, 469 ms lang, Blinder von 'na na na na' klingt noch 469 ms aus
+Alter Effekt: langsames Füllen LED für LED, alle 5 s eine neue Farbe. Eine Achtel vor dem Stopp (51,875) blitzt ein schneller Blinder (warmweiß, alle Geräte) und klingt in 1 Beat ins Schwarz des Stopps ab.</t>
         </is>
       </c>
       <c r="D198" s="12" t="n"/>
@@ -3038,7 +3072,7 @@
       </c>
       <c r="J198" s="7" t="n"/>
     </row>
-    <row r="199" hidden="1" outlineLevel="2">
+    <row r="199" outlineLevel="2">
       <c r="A199" s="4" t="n">
         <v>49.25</v>
       </c>
@@ -3050,7 +3084,7 @@
       <c r="G199" s="6" t="n"/>
       <c r="J199" s="7" t="n"/>
     </row>
-    <row r="200" hidden="1" outlineLevel="2">
+    <row r="200" outlineLevel="2">
       <c r="A200" s="4" t="n">
         <v>49.5</v>
       </c>
@@ -3062,7 +3096,7 @@
       <c r="G200" s="6" t="n"/>
       <c r="J200" s="7" t="n"/>
     </row>
-    <row r="201" hidden="1" outlineLevel="2">
+    <row r="201" outlineLevel="2">
       <c r="A201" s="4" t="n">
         <v>49.75</v>
       </c>
@@ -3074,7 +3108,7 @@
       <c r="G201" s="6" t="n"/>
       <c r="J201" s="7" t="n"/>
     </row>
-    <row r="202" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="202" outlineLevel="1" collapsed="1">
       <c r="A202" s="4" t="n">
         <v>50</v>
       </c>
@@ -3122,7 +3156,7 @@
       <c r="G205" s="6" t="n"/>
       <c r="J205" s="7" t="n"/>
     </row>
-    <row r="206" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="206" outlineLevel="1">
       <c r="A206" s="4" t="n">
         <v>51</v>
       </c>
@@ -3134,7 +3168,7 @@
       <c r="G206" s="6" t="n"/>
       <c r="J206" s="7" t="n"/>
     </row>
-    <row r="207" hidden="1" outlineLevel="2">
+    <row r="207" outlineLevel="2">
       <c r="A207" s="4" t="n">
         <v>51.25</v>
       </c>
@@ -3146,7 +3180,7 @@
       <c r="G207" s="6" t="n"/>
       <c r="J207" s="7" t="n"/>
     </row>
-    <row r="208" hidden="1" outlineLevel="2">
+    <row r="208" outlineLevel="2">
       <c r="A208" s="4" t="n">
         <v>51.5</v>
       </c>
@@ -3158,13 +3192,21 @@
       <c r="G208" s="6" t="n"/>
       <c r="J208" s="7" t="n"/>
     </row>
-    <row r="209" hidden="1" outlineLevel="2">
+    <row r="209" outlineLevel="2" ht="28.8" customHeight="1">
       <c r="A209" s="4" t="n">
         <v>51.75</v>
       </c>
       <c r="B209" s="5" t="n"/>
-      <c r="C209" s="6" t="n"/>
-      <c r="D209" s="12" t="n"/>
+      <c r="C209" s="6" t="inlineStr">
+        <is>
+          <t>Blinder auf 51,875 (eine Achtel vor dem Stopp), klingt in 1 Beat in den Stopp aus</t>
+        </is>
+      </c>
+      <c r="D209" s="12" t="inlineStr">
+        <is>
+          <t>den folgenden Blinder schon etwas früher, hier bei 51,875</t>
+        </is>
+      </c>
       <c r="E209" s="10" t="n"/>
       <c r="F209" s="10" t="n"/>
       <c r="G209" s="6" t="n"/>
@@ -3181,12 +3223,16 @@
       </c>
       <c r="C210" s="6" t="inlineStr">
         <is>
-          <t>progBlack(1875, 50)
-Ausgabe: Blinder bei 0 ms, 469 ms lang
-1 Takt Stille. Auf den Stopp-Schlag blitzt ein schneller Blinder (warmweiß, alle Geräte) und klingt in 1 Beat ins Schwarz ab.</t>
-        </is>
-      </c>
-      <c r="D210" s="12" t="n"/>
+          <t>progBlack(1875, 12)
+Ausgabe: Blinder von 'verse 2' klingt noch 235 ms aus
+1 Takt Stille (der Blinder davor klingt noch kurz aus).</t>
+        </is>
+      </c>
+      <c r="D210" s="12" t="inlineStr">
+        <is>
+          <t>den blinder hier raus weil er jetzt schon bei 51,875 kommt</t>
+        </is>
+      </c>
       <c r="E210" s="10" t="n">
         <v>0</v>
       </c>
@@ -3448,7 +3494,7 @@
       <c r="G229" s="6" t="n"/>
       <c r="J229" s="7" t="n"/>
     </row>
-    <row r="230" collapsed="1" ht="100.8" customHeight="1">
+    <row r="230" ht="100.8" customHeight="1">
       <c r="A230" s="4" t="n">
         <v>57</v>
       </c>
@@ -3459,10 +3505,10 @@
       </c>
       <c r="C230" s="6" t="inlineStr">
         <is>
-          <t>progWaterRipple(15000, 60, 50, true, false)
-Text (Matrix): "A B C D E": A 1 x, B 1 x, C 1 x, D 1 x, E 9 x 469 ms, ein Durchlauf 6097 ms (über der Szene)
-   ab 12188 ms bis 14531 ms, darunter 15 %
-Alter Effekt: Wasserringe an zufälligen Stellen, mit Farbverlauf. Ab Takt 6,5 des Parts (Beat 26) erscheinen auf der Matrix A, B, C, D, E in Weiß, je ein Viertel lang, über dem gedimmten Effekt.</t>
+          <t>progWaterRipple(15000, 14, 50, true, false)
+Text (Matrix): "A B C D E": A 1 x, B 1 x, C 1 x, D 1 x, E 9 x 469 ms, ein Durchlauf 6097 ms (über Szene und Ebene, ab 12188 ms bis 14531 ms, darunter 15 %)
+   Fenster 1: ab 14531 ms bis 18281 ms (blendet im nächsten Part aus), klingt 938 ms ab
+Alter Effekt: Wasserringe an zufälligen Stellen, mit Farbverlauf. Ab Takt 6,5 des Parts (Beat 26) erscheinen auf der Matrix A, B, C, D, E in Weiß, je ein Viertel lang, über dem gedimmten Effekt. Auf der letzten Viertel (64,75) steht FUCK YOU schwarz ausgestanzt und bleibt bis in den Chorus.</t>
         </is>
       </c>
       <c r="D230" s="12" t="n"/>
@@ -3480,7 +3526,7 @@
       </c>
       <c r="J230" s="7" t="n"/>
     </row>
-    <row r="231" hidden="1" outlineLevel="2">
+    <row r="231" outlineLevel="2">
       <c r="A231" s="4" t="n">
         <v>57.25</v>
       </c>
@@ -3492,7 +3538,7 @@
       <c r="G231" s="6" t="n"/>
       <c r="J231" s="7" t="n"/>
     </row>
-    <row r="232" hidden="1" outlineLevel="2">
+    <row r="232" outlineLevel="2">
       <c r="A232" s="4" t="n">
         <v>57.5</v>
       </c>
@@ -3504,7 +3550,7 @@
       <c r="G232" s="6" t="n"/>
       <c r="J232" s="7" t="n"/>
     </row>
-    <row r="233" hidden="1" outlineLevel="2">
+    <row r="233" outlineLevel="2">
       <c r="A233" s="4" t="n">
         <v>57.75</v>
       </c>
@@ -3516,7 +3562,7 @@
       <c r="G233" s="6" t="n"/>
       <c r="J233" s="7" t="n"/>
     </row>
-    <row r="234" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="234" outlineLevel="1" collapsed="1">
       <c r="A234" s="4" t="n">
         <v>58</v>
       </c>
@@ -3564,7 +3610,7 @@
       <c r="G237" s="6" t="n"/>
       <c r="J237" s="7" t="n"/>
     </row>
-    <row r="238" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="238" outlineLevel="1" collapsed="1">
       <c r="A238" s="4" t="n">
         <v>59</v>
       </c>
@@ -3612,7 +3658,7 @@
       <c r="G241" s="6" t="n"/>
       <c r="J241" s="7" t="n"/>
     </row>
-    <row r="242" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="242" outlineLevel="1" collapsed="1">
       <c r="A242" s="4" t="n">
         <v>60</v>
       </c>
@@ -3660,7 +3706,7 @@
       <c r="G245" s="6" t="n"/>
       <c r="J245" s="7" t="n"/>
     </row>
-    <row r="246" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="246" outlineLevel="1" collapsed="1">
       <c r="A246" s="4" t="n">
         <v>61</v>
       </c>
@@ -3708,7 +3754,7 @@
       <c r="G249" s="6" t="n"/>
       <c r="J249" s="7" t="n"/>
     </row>
-    <row r="250" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="250" outlineLevel="1" collapsed="1">
       <c r="A250" s="4" t="n">
         <v>62</v>
       </c>
@@ -3756,7 +3802,7 @@
       <c r="G253" s="6" t="n"/>
       <c r="J253" s="7" t="n"/>
     </row>
-    <row r="254" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="254" outlineLevel="1" collapsed="1">
       <c r="A254" s="4" t="n">
         <v>63</v>
       </c>
@@ -3804,7 +3850,7 @@
       <c r="G257" s="6" t="n"/>
       <c r="J257" s="7" t="n"/>
     </row>
-    <row r="258" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="258" outlineLevel="1">
       <c r="A258" s="4" t="n">
         <v>64</v>
       </c>
@@ -3816,7 +3862,7 @@
       <c r="G258" s="6" t="n"/>
       <c r="J258" s="7" t="n"/>
     </row>
-    <row r="259" hidden="1" outlineLevel="2">
+    <row r="259" outlineLevel="2">
       <c r="A259" s="4" t="n">
         <v>64.25</v>
       </c>
@@ -3828,7 +3874,7 @@
       <c r="G259" s="6" t="n"/>
       <c r="J259" s="7" t="n"/>
     </row>
-    <row r="260" hidden="1" outlineLevel="2">
+    <row r="260" outlineLevel="2">
       <c r="A260" s="4" t="n">
         <v>64.5</v>
       </c>
@@ -3840,19 +3886,28 @@
       <c r="G260" s="6" t="n"/>
       <c r="J260" s="7" t="n"/>
     </row>
-    <row r="261" hidden="1" outlineLevel="2">
+    <row r="261" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A261" s="4" t="n">
         <v>64.75</v>
       </c>
       <c r="B261" s="5" t="n"/>
-      <c r="C261" s="6" t="n"/>
-      <c r="D261" s="12" t="n"/>
+      <c r="C261" s="6" t="inlineStr">
+        <is>
+          <t>FUCK YOU schwarz ausgestanzt schon eine Viertel vor dem Chorus, 1,5 Takte voll, blendet im Chorus bis 66,75 aus</t>
+        </is>
+      </c>
+      <c r="D261" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E261" s="10" t="n"/>
       <c r="F261" s="10" t="n"/>
       <c r="G261" s="6" t="n"/>
       <c r="J261" s="7" t="n"/>
     </row>
-    <row r="262" collapsed="1" ht="86.40000000000001" customHeight="1">
+    <row r="262" ht="86.40000000000001" customHeight="1">
       <c r="A262" s="4" t="n">
         <v>65</v>
       </c>
@@ -3863,13 +3918,17 @@
       </c>
       <c r="C262" s="6" t="inlineStr">
         <is>
-          <t>progFullColors(15000, 65, 469)
-Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (über der Szene)
-   ab 0 ms bis 3750 ms, klingt 3750 ms ab, darunter 15 %
-Alter Effekt wie Chorus 1: pro Beat eine neue Farbe. Auf der Matrix steht auf den Einsatz FUCK YOU in Weiß und blendet über 2 Takte aus, der Effekt darunter kommt dabei wieder hoch.</t>
-        </is>
-      </c>
-      <c r="D262" s="6" t="n"/>
+          <t>progFullColors(15000, 15, 469)
+Text (Matrix): "FUCK_YOU FUCK_OFF": FUCK_YOU 29 x, FUCK_OFF 35 x 469 ms, ein Durchlauf 30016 ms (ausgestanzt aus der Szene)
+   Fenster 1: ab 0 ms bis 3281 ms, Fenster 2: ab 7031 ms bis 10781 ms, Fenster 3: ab 13594 ms bis 17344 ms (blendet im nächsten Part aus), klingt 938 ms ab
+Alter Effekt wie Chorus 1: pro Beat eine neue Farbe. Auf der Matrix FUCK YOU schwarz ausgestanzt in der Farbfläche: das von der Viertel davor steht bis 66,25 und blendet bis 66,75 aus, dann auf 68,75 FUCK YOU und auf 72,25 FUCK OFF, je 1,5 Takte voll und 0,5 Takte ausblendend.</t>
+        </is>
+      </c>
+      <c r="D262" s="6" t="inlineStr">
+        <is>
+          <t>text beginnt schon in der Zeile vorher</t>
+        </is>
+      </c>
       <c r="E262" s="10" t="n">
         <v>5</v>
       </c>
@@ -3884,7 +3943,7 @@
       </c>
       <c r="J262" s="7" t="n"/>
     </row>
-    <row r="263" hidden="1" outlineLevel="2">
+    <row r="263" outlineLevel="2">
       <c r="A263" s="4" t="n">
         <v>65.25</v>
       </c>
@@ -3896,7 +3955,7 @@
       <c r="G263" s="6" t="n"/>
       <c r="J263" s="7" t="n"/>
     </row>
-    <row r="264" hidden="1" outlineLevel="2">
+    <row r="264" outlineLevel="2">
       <c r="A264" s="4" t="n">
         <v>65.5</v>
       </c>
@@ -3908,7 +3967,7 @@
       <c r="G264" s="6" t="n"/>
       <c r="J264" s="7" t="n"/>
     </row>
-    <row r="265" hidden="1" outlineLevel="2">
+    <row r="265" outlineLevel="2">
       <c r="A265" s="4" t="n">
         <v>65.75</v>
       </c>
@@ -3920,7 +3979,7 @@
       <c r="G265" s="6" t="n"/>
       <c r="J265" s="7" t="n"/>
     </row>
-    <row r="266" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="266" outlineLevel="1" collapsed="1">
       <c r="A266" s="4" t="n">
         <v>66</v>
       </c>
@@ -3968,7 +4027,7 @@
       <c r="G269" s="6" t="n"/>
       <c r="J269" s="7" t="n"/>
     </row>
-    <row r="270" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="270" outlineLevel="1" collapsed="1">
       <c r="A270" s="4" t="n">
         <v>67</v>
       </c>
@@ -4016,7 +4075,7 @@
       <c r="G273" s="6" t="n"/>
       <c r="J273" s="7" t="n"/>
     </row>
-    <row r="274" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="274" outlineLevel="1">
       <c r="A274" s="4" t="n">
         <v>68</v>
       </c>
@@ -4028,7 +4087,7 @@
       <c r="G274" s="6" t="n"/>
       <c r="J274" s="7" t="n"/>
     </row>
-    <row r="275" hidden="1" outlineLevel="2">
+    <row r="275" outlineLevel="2">
       <c r="A275" s="4" t="n">
         <v>68.25</v>
       </c>
@@ -4040,7 +4099,7 @@
       <c r="G275" s="6" t="n"/>
       <c r="J275" s="7" t="n"/>
     </row>
-    <row r="276" hidden="1" outlineLevel="2">
+    <row r="276" outlineLevel="2">
       <c r="A276" s="4" t="n">
         <v>68.5</v>
       </c>
@@ -4052,19 +4111,28 @@
       <c r="G276" s="6" t="n"/>
       <c r="J276" s="7" t="n"/>
     </row>
-    <row r="277" hidden="1" outlineLevel="2">
+    <row r="277" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A277" s="4" t="n">
         <v>68.75</v>
       </c>
       <c r="B277" s="5" t="n"/>
-      <c r="C277" s="6" t="n"/>
-      <c r="D277" s="6" t="n"/>
+      <c r="C277" s="6" t="inlineStr">
+        <is>
+          <t>FUCK YOU schwarz ausgestanzt, 1,5 Takte voll, dann bis 70,75 ausblenden</t>
+        </is>
+      </c>
+      <c r="D277" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E277" s="10" t="n"/>
       <c r="F277" s="10" t="n"/>
       <c r="G277" s="6" t="n"/>
       <c r="J277" s="7" t="n"/>
     </row>
-    <row r="278" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="278" outlineLevel="1" collapsed="1">
       <c r="A278" s="4" t="n">
         <v>69</v>
       </c>
@@ -4112,7 +4180,7 @@
       <c r="G281" s="6" t="n"/>
       <c r="J281" s="7" t="n"/>
     </row>
-    <row r="282" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="282" outlineLevel="1" collapsed="1">
       <c r="A282" s="4" t="n">
         <v>70</v>
       </c>
@@ -4160,7 +4228,7 @@
       <c r="G285" s="6" t="n"/>
       <c r="J285" s="7" t="n"/>
     </row>
-    <row r="286" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="286" outlineLevel="1" collapsed="1">
       <c r="A286" s="4" t="n">
         <v>71</v>
       </c>
@@ -4208,7 +4276,7 @@
       <c r="G289" s="6" t="n"/>
       <c r="J289" s="7" t="n"/>
     </row>
-    <row r="290" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="290" outlineLevel="1">
       <c r="A290" s="4" t="n">
         <v>72</v>
       </c>
@@ -4220,19 +4288,28 @@
       <c r="G290" s="6" t="n"/>
       <c r="J290" s="7" t="n"/>
     </row>
-    <row r="291" hidden="1" outlineLevel="2">
+    <row r="291" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A291" s="4" t="n">
         <v>72.25</v>
       </c>
       <c r="B291" s="5" t="n"/>
-      <c r="C291" s="6" t="n"/>
-      <c r="D291" s="6" t="n"/>
+      <c r="C291" s="6" t="inlineStr">
+        <is>
+          <t>FUCK OFF schwarz ausgestanzt, 1,5 Takte voll, blendet im na na na na bis 74,25 aus</t>
+        </is>
+      </c>
+      <c r="D291" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK OFF": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E291" s="10" t="n"/>
       <c r="F291" s="10" t="n"/>
       <c r="G291" s="6" t="n"/>
       <c r="J291" s="7" t="n"/>
     </row>
-    <row r="292" hidden="1" outlineLevel="2">
+    <row r="292" outlineLevel="2">
       <c r="A292" s="4" t="n">
         <v>72.5</v>
       </c>
@@ -4244,7 +4321,7 @@
       <c r="G292" s="6" t="n"/>
       <c r="J292" s="7" t="n"/>
     </row>
-    <row r="293" hidden="1" outlineLevel="2">
+    <row r="293" outlineLevel="2">
       <c r="A293" s="4" t="n">
         <v>72.75</v>
       </c>
@@ -4256,7 +4333,7 @@
       <c r="G293" s="6" t="n"/>
       <c r="J293" s="7" t="n"/>
     </row>
-    <row r="294" collapsed="1" ht="100.8" customHeight="1">
+    <row r="294" ht="100.8" customHeight="1">
       <c r="A294" s="4" t="n">
         <v>73</v>
       </c>
@@ -4267,13 +4344,17 @@
       </c>
       <c r="C294" s="6" t="inlineStr">
         <is>
-          <t>progSternNeu(15000, 469, 70, 5, 26, 5, true, 4)
-Text (Matrix): "A B C D E": A 1 x, B 1 x, C 1 x, D 1 x, E 9 x 469 ms, ein Durchlauf 6097 ms (über der Szene)
-   ab 12188 ms bis 14531 ms, darunter 15 %
-Alter Effekt: drehender Stern, diesmal wandernd. Ab Takt 6,5 des Parts (Beat 26) erscheinen auf der Matrix A, B, C, D, E in Weiß, je ein Viertel lang, über dem gedimmten Effekt.</t>
-        </is>
-      </c>
-      <c r="D294" s="6" t="n"/>
+          <t>progSternNeu(15000, 469, 16, 5, 26, 5, true, 4)
+Text (Matrix): "A B C D E": A 1 x, B 1 x, C 1 x, D 1 x, E 9 x 469 ms, ein Durchlauf 6097 ms (über Szene und Ebene, ab 12188 ms bis 14531 ms, darunter 15 %)
+   Fenster 1: ab 0 ms bis 2344 ms, Fenster 2: ab 14531 ms bis 18281 ms (blendet im nächsten Part aus), klingt 938 ms ab
+Alter Effekt: drehender Stern, diesmal wandernd. Das FUCK OFF aus dem Chorus steht noch 3 Beats und blendet bis 74,25 aus. Ab Takt 6,5 des Parts (Beat 26) erscheinen auf der Matrix A, B, C, D, E in Weiß, je ein Viertel lang, über dem gedimmten Effekt; auf der letzten Viertel (80,75) FUCK YOU schwarz ausgestanzt bis in den Chorus.</t>
+        </is>
+      </c>
+      <c r="D294" s="6" t="inlineStr">
+        <is>
+          <t>text s.o.</t>
+        </is>
+      </c>
       <c r="E294" s="10" t="n">
         <v>4</v>
       </c>
@@ -4288,7 +4369,7 @@
       </c>
       <c r="J294" s="7" t="n"/>
     </row>
-    <row r="295" hidden="1" outlineLevel="2">
+    <row r="295" outlineLevel="2">
       <c r="A295" s="4" t="n">
         <v>73.25</v>
       </c>
@@ -4300,7 +4381,7 @@
       <c r="G295" s="6" t="n"/>
       <c r="J295" s="7" t="n"/>
     </row>
-    <row r="296" hidden="1" outlineLevel="2">
+    <row r="296" outlineLevel="2">
       <c r="A296" s="4" t="n">
         <v>73.5</v>
       </c>
@@ -4312,7 +4393,7 @@
       <c r="G296" s="6" t="n"/>
       <c r="J296" s="7" t="n"/>
     </row>
-    <row r="297" hidden="1" outlineLevel="2">
+    <row r="297" outlineLevel="2">
       <c r="A297" s="4" t="n">
         <v>73.75</v>
       </c>
@@ -4324,7 +4405,7 @@
       <c r="G297" s="6" t="n"/>
       <c r="J297" s="7" t="n"/>
     </row>
-    <row r="298" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="298" outlineLevel="1" collapsed="1">
       <c r="A298" s="4" t="n">
         <v>74</v>
       </c>
@@ -4372,7 +4453,7 @@
       <c r="G301" s="6" t="n"/>
       <c r="J301" s="7" t="n"/>
     </row>
-    <row r="302" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="302" outlineLevel="1" collapsed="1">
       <c r="A302" s="4" t="n">
         <v>75</v>
       </c>
@@ -4420,7 +4501,7 @@
       <c r="G305" s="6" t="n"/>
       <c r="J305" s="7" t="n"/>
     </row>
-    <row r="306" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="306" outlineLevel="1" collapsed="1">
       <c r="A306" s="4" t="n">
         <v>76</v>
       </c>
@@ -4468,7 +4549,7 @@
       <c r="G309" s="6" t="n"/>
       <c r="J309" s="7" t="n"/>
     </row>
-    <row r="310" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="310" outlineLevel="1" collapsed="1">
       <c r="A310" s="4" t="n">
         <v>77</v>
       </c>
@@ -4516,7 +4597,7 @@
       <c r="G313" s="6" t="n"/>
       <c r="J313" s="7" t="n"/>
     </row>
-    <row r="314" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="314" outlineLevel="1" collapsed="1">
       <c r="A314" s="4" t="n">
         <v>78</v>
       </c>
@@ -4564,7 +4645,7 @@
       <c r="G317" s="6" t="n"/>
       <c r="J317" s="7" t="n"/>
     </row>
-    <row r="318" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="318" outlineLevel="1" collapsed="1">
       <c r="A318" s="4" t="n">
         <v>79</v>
       </c>
@@ -4612,7 +4693,7 @@
       <c r="G321" s="6" t="n"/>
       <c r="J321" s="7" t="n"/>
     </row>
-    <row r="322" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="322" outlineLevel="1">
       <c r="A322" s="4" t="n">
         <v>80</v>
       </c>
@@ -4624,7 +4705,7 @@
       <c r="G322" s="6" t="n"/>
       <c r="J322" s="7" t="n"/>
     </row>
-    <row r="323" hidden="1" outlineLevel="2">
+    <row r="323" outlineLevel="2">
       <c r="A323" s="4" t="n">
         <v>80.25</v>
       </c>
@@ -4636,7 +4717,7 @@
       <c r="G323" s="6" t="n"/>
       <c r="J323" s="7" t="n"/>
     </row>
-    <row r="324" hidden="1" outlineLevel="2">
+    <row r="324" outlineLevel="2">
       <c r="A324" s="4" t="n">
         <v>80.5</v>
       </c>
@@ -4648,19 +4729,28 @@
       <c r="G324" s="6" t="n"/>
       <c r="J324" s="7" t="n"/>
     </row>
-    <row r="325" hidden="1" outlineLevel="2">
+    <row r="325" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A325" s="4" t="n">
         <v>80.75</v>
       </c>
       <c r="B325" s="5" t="n"/>
-      <c r="C325" s="6" t="n"/>
-      <c r="D325" s="6" t="n"/>
+      <c r="C325" s="6" t="inlineStr">
+        <is>
+          <t>FUCK YOU schwarz ausgestanzt schon eine Viertel vor dem Chorus, 1,5 Takte voll, blendet im Chorus bis 82,75 aus</t>
+        </is>
+      </c>
+      <c r="D325" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E325" s="10" t="n"/>
       <c r="F325" s="10" t="n"/>
       <c r="G325" s="6" t="n"/>
       <c r="J325" s="7" t="n"/>
     </row>
-    <row r="326" collapsed="1" ht="72" customHeight="1">
+    <row r="326" ht="72" customHeight="1">
       <c r="A326" s="4" t="n">
         <v>81</v>
       </c>
@@ -4671,13 +4761,17 @@
       </c>
       <c r="C326" s="6" t="inlineStr">
         <is>
-          <t>progFastBlingBling(15000, 4, 75)
-Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (über der Szene)
-   ab 0 ms bis 3750 ms, klingt 3750 ms ab, darunter 15 %
-Alter Effekt: schnelle Einzelblitze für den letzten Chorus. Auf der Matrix steht auf den Einsatz FUCK YOU in Weiß und blendet über 2 Takte aus.</t>
-        </is>
-      </c>
-      <c r="D326" s="6" t="n"/>
+          <t>progFastBlingBling(15000, 4, 17)
+Text (Matrix): "FUCK_YOU FUCK_OFF": FUCK_YOU 29 x, FUCK_OFF 35 x 469 ms, ein Durchlauf 30016 ms (ausgestanzt aus der Szene)
+   Fenster 1: ab 0 ms bis 3281 ms, Fenster 2: ab 7031 ms bis 10781 ms, Fenster 3: ab 13594 ms bis 17344 ms (blendet im nächsten Part aus), klingt 938 ms ab
+Alter Effekt: schnelle Einzelblitze für den letzten Chorus. Auf der Matrix FUCK YOU schwarz ausgestanzt aus den Blitzen: das von der Viertel davor steht bis 82,25 und blendet bis 82,75 aus, dann auf 84,75 FUCK YOU und auf 88,25 FUCK OFF, je 1,5 Takte voll und 0,5 Takte ausblendend.</t>
+        </is>
+      </c>
+      <c r="D326" s="6" t="inlineStr">
+        <is>
+          <t>text beginnt schon in der Zeile vorher</t>
+        </is>
+      </c>
       <c r="E326" s="10" t="n">
         <v>5</v>
       </c>
@@ -4692,7 +4786,7 @@
       </c>
       <c r="J326" s="7" t="n"/>
     </row>
-    <row r="327" hidden="1" outlineLevel="2">
+    <row r="327" outlineLevel="2">
       <c r="A327" s="4" t="n">
         <v>81.25</v>
       </c>
@@ -4704,7 +4798,7 @@
       <c r="G327" s="6" t="n"/>
       <c r="J327" s="7" t="n"/>
     </row>
-    <row r="328" hidden="1" outlineLevel="2">
+    <row r="328" outlineLevel="2">
       <c r="A328" s="4" t="n">
         <v>81.5</v>
       </c>
@@ -4716,7 +4810,7 @@
       <c r="G328" s="6" t="n"/>
       <c r="J328" s="7" t="n"/>
     </row>
-    <row r="329" hidden="1" outlineLevel="2">
+    <row r="329" outlineLevel="2">
       <c r="A329" s="4" t="n">
         <v>81.75</v>
       </c>
@@ -4728,7 +4822,7 @@
       <c r="G329" s="6" t="n"/>
       <c r="J329" s="7" t="n"/>
     </row>
-    <row r="330" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="330" outlineLevel="1" collapsed="1">
       <c r="A330" s="4" t="n">
         <v>82</v>
       </c>
@@ -4776,7 +4870,7 @@
       <c r="G333" s="6" t="n"/>
       <c r="J333" s="7" t="n"/>
     </row>
-    <row r="334" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="334" outlineLevel="1" collapsed="1">
       <c r="A334" s="4" t="n">
         <v>83</v>
       </c>
@@ -4824,7 +4918,7 @@
       <c r="G337" s="6" t="n"/>
       <c r="J337" s="7" t="n"/>
     </row>
-    <row r="338" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="338" outlineLevel="1">
       <c r="A338" s="4" t="n">
         <v>84</v>
       </c>
@@ -4836,7 +4930,7 @@
       <c r="G338" s="6" t="n"/>
       <c r="J338" s="7" t="n"/>
     </row>
-    <row r="339" hidden="1" outlineLevel="2">
+    <row r="339" outlineLevel="2">
       <c r="A339" s="4" t="n">
         <v>84.25</v>
       </c>
@@ -4848,7 +4942,7 @@
       <c r="G339" s="6" t="n"/>
       <c r="J339" s="7" t="n"/>
     </row>
-    <row r="340" hidden="1" outlineLevel="2">
+    <row r="340" outlineLevel="2">
       <c r="A340" s="4" t="n">
         <v>84.5</v>
       </c>
@@ -4860,19 +4954,28 @@
       <c r="G340" s="6" t="n"/>
       <c r="J340" s="7" t="n"/>
     </row>
-    <row r="341" hidden="1" outlineLevel="2">
+    <row r="341" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A341" s="4" t="n">
         <v>84.75</v>
       </c>
       <c r="B341" s="5" t="n"/>
-      <c r="C341" s="6" t="n"/>
-      <c r="D341" s="6" t="n"/>
+      <c r="C341" s="6" t="inlineStr">
+        <is>
+          <t>FUCK YOU schwarz ausgestanzt, 1,5 Takte voll, dann bis 86,75 ausblenden</t>
+        </is>
+      </c>
+      <c r="D341" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK YOU": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E341" s="10" t="n"/>
       <c r="F341" s="10" t="n"/>
       <c r="G341" s="6" t="n"/>
       <c r="J341" s="7" t="n"/>
     </row>
-    <row r="342" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="342" outlineLevel="1" collapsed="1">
       <c r="A342" s="4" t="n">
         <v>85</v>
       </c>
@@ -4920,7 +5023,7 @@
       <c r="G345" s="6" t="n"/>
       <c r="J345" s="7" t="n"/>
     </row>
-    <row r="346" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="346" outlineLevel="1" collapsed="1">
       <c r="A346" s="4" t="n">
         <v>86</v>
       </c>
@@ -4968,7 +5071,7 @@
       <c r="G349" s="6" t="n"/>
       <c r="J349" s="7" t="n"/>
     </row>
-    <row r="350" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="350" outlineLevel="1" collapsed="1">
       <c r="A350" s="4" t="n">
         <v>87</v>
       </c>
@@ -5016,7 +5119,7 @@
       <c r="G353" s="6" t="n"/>
       <c r="J353" s="7" t="n"/>
     </row>
-    <row r="354" hidden="1" outlineLevel="1" collapsed="1">
+    <row r="354" outlineLevel="1">
       <c r="A354" s="4" t="n">
         <v>88</v>
       </c>
@@ -5028,19 +5131,28 @@
       <c r="G354" s="6" t="n"/>
       <c r="J354" s="7" t="n"/>
     </row>
-    <row r="355" hidden="1" outlineLevel="2">
+    <row r="355" outlineLevel="2" ht="43.2" customHeight="1">
       <c r="A355" s="4" t="n">
         <v>88.25</v>
       </c>
       <c r="B355" s="5" t="n"/>
-      <c r="C355" s="6" t="n"/>
-      <c r="D355" s="6" t="n"/>
+      <c r="C355" s="6" t="inlineStr">
+        <is>
+          <t>FUCK OFF schwarz ausgestanzt, 1,5 Takte voll, blendet in den Triolen bis 90,25 aus</t>
+        </is>
+      </c>
+      <c r="D355" s="6" t="inlineStr">
+        <is>
+          <t>Text (Matrix): "FUCK OFF": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+nach 1,5 Takten (über 0,5 Takte) ausblenden</t>
+        </is>
+      </c>
       <c r="E355" s="10" t="n"/>
       <c r="F355" s="10" t="n"/>
       <c r="G355" s="6" t="n"/>
       <c r="J355" s="7" t="n"/>
     </row>
-    <row r="356" hidden="1" outlineLevel="2">
+    <row r="356" outlineLevel="2">
       <c r="A356" s="4" t="n">
         <v>88.5</v>
       </c>
@@ -5052,7 +5164,7 @@
       <c r="G356" s="6" t="n"/>
       <c r="J356" s="7" t="n"/>
     </row>
-    <row r="357" hidden="1" outlineLevel="2">
+    <row r="357" outlineLevel="2">
       <c r="A357" s="4" t="n">
         <v>88.75</v>
       </c>
@@ -5075,11 +5187,17 @@
       </c>
       <c r="C358" s="6" t="inlineStr">
         <is>
-          <t>progStrobo(4688, 80, 469, 255, 255, 255)
-Weißer Strobo im Viertel-Raster: ein Viertel lang an, das nächste Viertel aus (469 ms), auf allen Geräten gleich.</t>
-        </is>
-      </c>
-      <c r="D358" s="11" t="n"/>
+          <t>progStrobo(4688, 18, 469, 255, 255, 255)
+Text (Matrix): "FUCK OFF": steht durchgehend, ohne Pulsieren (ausgestanzt aus der Szene)
+   Fenster 1: ab 0 ms bis 2344 ms, klingt 938 ms ab
+Das FUCK OFF aus dem Chorus steht noch 3 Beats schwarz ausgestanzt im Strobo und blendet bis 90,25 aus. Weißer Strobo im Viertel-Raster: ein Viertel lang an, das nächste Viertel aus (469 ms), auf allen Geräten gleich.</t>
+        </is>
+      </c>
+      <c r="D358" s="6" t="inlineStr">
+        <is>
+          <t>text s.o.</t>
+        </is>
+      </c>
       <c r="E358" s="10" t="n">
         <v>5</v>
       </c>

</xml_diff>